<commit_message>
Fix the Form 5 basis text, which still printed the old lookup order
The values flipped with the direction, but the "判定依據" string in
export_xlsx.py still read (base − comparable) × step, so every Form 5
percentage cell carried a note contradicting its own number: the FAR row
showed 6.25 while its comment derived (3−4)×6.25, i.e. −6.25. The note is
what a reviewer reads to check the cell, so a wrong one is worse than none.

Regenerated versions 2-4, finalVersion, the previews and the field map.
Checked afterwards that all 762 lookup expressions in the workbooks and
all 114 in the HTML now evaluate to the value they sit next to.
</commit_message>
<xml_diff>
--- a/output/finalVersion/表5-1_影響地價區域因素分析明細表_已填.xlsx
+++ b/output/finalVersion/表5-1_影響地價區域因素分析明細表_已填.xlsx
@@ -1281,7 +1281,7 @@
         <t>【AI判定】容積率（P002-00 修正百分比）
 填寫值：6.25
 資料來源：比準地 P001-00 普通(3) ／ P002-00 稍劣(4)
-判定依據：查表：共5級、最大±25.0%、級距6.25%；(3−4)×6.25 = +6.25
+判定依據：查表：共5級、最大±25.0%、級距6.25%；(4−3)×6.25 = +6.25
 基準表項目ID：shulin.regional.far</t>
       </text>
     </comment>
@@ -1605,7 +1605,7 @@
         <t>【AI判定】主要道路寬度（P002-00 修正百分比）
 填寫值：15.0
 資料來源：比準地 P001-00 優(1) ／ P002-00 劣(5)
-判定依據：查表：共5級、最大±15.0%、級距3.75%；(1−5)×3.75 = +15.00
+判定依據：查表：共5級、最大±15.0%、級距3.75%；(5−1)×3.75 = +15.00
 基準表項目ID：shulin.regional.main_road_width</t>
       </text>
     </comment>
@@ -1632,7 +1632,7 @@
         <t>【AI判定】主要道路寬度（P003-00 修正百分比）
 填寫值：11.25
 資料來源：比準地 P001-00 優(1) ／ P003-00 稍劣(4)
-判定依據：查表：共5級、最大±15.0%、級距3.75%；(1−4)×3.75 = +11.25
+判定依據：查表：共5級、最大±15.0%、級距3.75%；(4−1)×3.75 = +11.25
 基準表項目ID：shulin.regional.main_road_width</t>
       </text>
     </comment>
@@ -1659,7 +1659,7 @@
         <t>【AI判定】主要道路寬度（P004-00 修正百分比）
 填寫值：11.25
 資料來源：比準地 P001-00 優(1) ／ P004-00 稍劣(4)
-判定依據：查表：共5級、最大±15.0%、級距3.75%；(1−4)×3.75 = +11.25
+判定依據：查表：共5級、最大±15.0%、級距3.75%；(4−1)×3.75 = +11.25
 基準表項目ID：shulin.regional.main_road_width</t>
       </text>
     </comment>
@@ -1704,7 +1704,7 @@
         <t>【AI判定】區段內道路平均寬度（P002-00 修正百分比）
 填寫值：6.0
 資料來源：比準地 P001-00 普通(3) ／ P002-00 劣(5)
-判定依據：查表：共5級、最大±12.0%、級距3.0%；(3−5)×3.0 = +6.00
+判定依據：查表：共5級、最大±12.0%、級距3.0%；(5−3)×3.0 = +6.00
 基準表項目ID：shulin.regional.avg_road_width</t>
       </text>
     </comment>
@@ -1731,7 +1731,7 @@
         <t>【AI判定】區段內道路平均寬度（P003-00 修正百分比）
 填寫值：6.0
 資料來源：比準地 P001-00 普通(3) ／ P003-00 劣(5)
-判定依據：查表：共5級、最大±12.0%、級距3.0%；(3−5)×3.0 = +6.00
+判定依據：查表：共5級、最大±12.0%、級距3.0%；(5−3)×3.0 = +6.00
 基準表項目ID：shulin.regional.avg_road_width</t>
       </text>
     </comment>
@@ -1758,7 +1758,7 @@
         <t>【AI判定】區段內道路平均寬度（P004-00 修正百分比）
 填寫值：6.0
 資料來源：比準地 P001-00 普通(3) ／ P004-00 劣(5)
-判定依據：查表：共5級、最大±12.0%、級距3.0%；(3−5)×3.0 = +6.00
+判定依據：查表：共5級、最大±12.0%、級距3.0%；(5−3)×3.0 = +6.00
 基準表項目ID：shulin.regional.avg_road_width</t>
       </text>
     </comment>
@@ -1803,7 +1803,7 @@
         <t>【AI判定】接近大型車站之程度（P002-00 修正百分比）
 填寫值：-2.5
 資料來源：比準地 P001-00 稍優(2) ／ P002-00 優(1)
-判定依據：查表：共5級、最大±10.0%、級距2.5%；(2−1)×2.5 = -2.50
+判定依據：查表：共5級、最大±10.0%、級距2.5%；(1−2)×2.5 = -2.50
 基準表項目ID：shulin.regional.near_station</t>
       </text>
     </comment>
@@ -1956,7 +1956,7 @@
         <t>【AI判定】站牌之接近程度或密集程度（P004-00 修正百分比）
 填寫值：1.0
 資料來源：比準地 P001-00 優(1) ／ P004-00 稍優(2)
-判定依據：查表：共5級、最大±4.0%、級距1.0%；(1−2)×1.0 = +1.00
+判定依據：查表：共5級、最大±4.0%、級距1.0%；(2−1)×1.0 = +1.00
 基準表項目ID：shulin.regional.near_busstop</t>
       </text>
     </comment>
@@ -2055,7 +2055,7 @@
         <t>【AI判定】交流道之有無及接近交流道之程度（P004-00 修正百分比）
 填寫值：1.0
 資料來源：比準地 P001-00 稍劣(4) ／ P004-00 劣(5)
-判定依據：查表：共5級、最大±4.0%、級距1.0%；(4−5)×1.0 = +1.00
+判定依據：查表：共5級、最大±4.0%、級距1.0%；(5−4)×1.0 = +1.00
 基準表項目ID：shulin.regional.near_interchange</t>
       </text>
     </comment>
@@ -2100,7 +2100,7 @@
         <t>【AI判定】區段內道路規劃及闢建程度（P002-00 修正百分比）
 填寫值：2.5
 資料來源：比準地 P001-00 稍優(2) ／ P002-00 普通(3)
-判定依據：查表：共5級、最大±10.0%、級距2.5%；(2−3)×2.5 = +2.50
+判定依據：查表：共5級、最大±10.0%、級距2.5%；(3−2)×2.5 = +2.50
 基準表項目ID：shulin.regional.road_dev</t>
       </text>
     </comment>
@@ -2127,7 +2127,7 @@
         <t>【AI判定】區段內道路規劃及闢建程度（P003-00 修正百分比）
 填寫值：-2.5
 資料來源：比準地 P001-00 稍優(2) ／ P003-00 優(1)
-判定依據：查表：共5級、最大±10.0%、級距2.5%；(2−1)×2.5 = -2.50
+判定依據：查表：共5級、最大±10.0%、級距2.5%；(1−2)×2.5 = -2.50
 基準表項目ID：shulin.regional.road_dev</t>
       </text>
     </comment>
@@ -2154,7 +2154,7 @@
         <t>【AI判定】區段內道路規劃及闢建程度（P004-00 修正百分比）
 填寫值：-2.5
 資料來源：比準地 P001-00 稍優(2) ／ P004-00 優(1)
-判定依據：查表：共5級、最大±10.0%、級距2.5%；(2−1)×2.5 = -2.50
+判定依據：查表：共5級、最大±10.0%、級距2.5%；(1−2)×2.5 = -2.50
 基準表項目ID：shulin.regional.road_dev</t>
       </text>
     </comment>
@@ -2973,7 +2973,7 @@
         <t>【AI判定】接近市場之程度（傳統市場、超級市場、超大型購物中心）（P002-00 修正百分比）
 填寫值：-4.0
 資料來源：比準地 P001-00 普通(3) ／ P002-00 優(1)
-判定依據：查表：共5級、最大±8.0%、級距2.0%；(3−1)×2.0 = -4.00
+判定依據：查表：共5級、最大±8.0%、級距2.0%；(1−3)×2.0 = -4.00
 基準表項目ID：shulin.regional.near_market</t>
       </text>
     </comment>
@@ -3000,7 +3000,7 @@
         <t>【AI判定】接近市場之程度（傳統市場、超級市場、超大型購物中心）（P003-00 修正百分比）
 填寫值：-4.0
 資料來源：比準地 P001-00 普通(3) ／ P003-00 優(1)
-判定依據：查表：共5級、最大±8.0%、級距2.0%；(3−1)×2.0 = -4.00
+判定依據：查表：共5級、最大±8.0%、級距2.0%；(1−3)×2.0 = -4.00
 基準表項目ID：shulin.regional.near_market</t>
       </text>
     </comment>
@@ -3027,7 +3027,7 @@
         <t>【AI判定】接近市場之程度（傳統市場、超級市場、超大型購物中心）（P004-00 修正百分比）
 填寫值：-2.0
 資料來源：比準地 P001-00 普通(3) ／ P004-00 稍優(2)
-判定依據：查表：共5級、最大±8.0%、級距2.0%；(3−2)×2.0 = -2.00
+判定依據：查表：共5級、最大±8.0%、級距2.0%；(2−3)×2.0 = -2.00
 基準表項目ID：shulin.regional.near_market</t>
       </text>
     </comment>
@@ -3126,7 +3126,7 @@
         <t>【AI判定】接近公園（里鄰公園、一般公園）、廣場、徒步區之程度（P004-00 修正百分比）
 填寫值：4.0
 資料來源：比準地 P001-00 優(1) ／ P004-00 普通(3)
-判定依據：查表：共5級、最大±8.0%、級距2.0%；(1−3)×2.0 = +4.00
+判定依據：查表：共5級、最大±8.0%、級距2.0%；(3−1)×2.0 = +4.00
 基準表項目ID：shulin.regional.near_park</t>
       </text>
     </comment>
@@ -3171,7 +3171,7 @@
         <t>【AI判定】接近觀光遊憩設施之程度（P002-00 修正百分比）
 填寫值：1.5
 資料來源：比準地 P001-00 優(1) ／ P002-00 稍優(2)
-判定依據：查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50
+判定依據：查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50
 基準表項目ID：shulin.regional.near_tourism</t>
       </text>
     </comment>
@@ -3198,7 +3198,7 @@
         <t>【AI判定】接近觀光遊憩設施之程度（P003-00 修正百分比）
 填寫值：1.5
 資料來源：比準地 P001-00 優(1) ／ P003-00 稍優(2)
-判定依據：查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50
+判定依據：查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50
 基準表項目ID：shulin.regional.near_tourism</t>
       </text>
     </comment>
@@ -3225,7 +3225,7 @@
         <t>【AI判定】接近觀光遊憩設施之程度（P004-00 修正百分比）
 填寫值：1.5
 資料來源：比準地 P001-00 優(1) ／ P004-00 稍優(2)
-判定依據：查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50
+判定依據：查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50
 基準表項目ID：shulin.regional.near_tourism</t>
       </text>
     </comment>
@@ -3270,7 +3270,7 @@
         <t>【AI判定】停車場地之便利程度（P002-00 修正百分比）
 填寫值：1.5
 資料來源：比準地 P001-00 優(1) ／ P002-00 稍優(2)
-判定依據：查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50
+判定依據：查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50
 基準表項目ID：shulin.regional.parking</t>
       </text>
     </comment>
@@ -3297,7 +3297,7 @@
         <t>【AI判定】停車場地之便利程度（P003-00 修正百分比）
 填寫值：1.5
 資料來源：比準地 P001-00 優(1) ／ P003-00 稍優(2)
-判定依據：查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50
+判定依據：查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50
 基準表項目ID：shulin.regional.parking</t>
       </text>
     </comment>
@@ -3594,7 +3594,7 @@
         <t>【AI判定】殯葬設施之有無及接近程度（P002-00 修正百分比）
 填寫值：-2.5
 資料來源：比準地 P001-00 劣(5) ／ P002-00 稍劣(4)
-判定依據：查表：共5級、最大±10.0%、級距2.5%；(5−4)×2.5 = -2.50
+判定依據：查表：共5級、最大±10.0%、級距2.5%；(4−5)×2.5 = -2.50
 基準表項目ID：shulin.regional.funeral_facility</t>
       </text>
     </comment>
@@ -3648,7 +3648,7 @@
         <t>【AI判定】殯葬設施之有無及接近程度（P004-00 修正百分比）
 填寫值：-2.5
 資料來源：比準地 P001-00 劣(5) ／ P004-00 稍劣(4)
-判定依據：查表：共5級、最大±10.0%、級距2.5%；(5−4)×2.5 = -2.50
+判定依據：查表：共5級、最大±10.0%、級距2.5%；(4−5)×2.5 = -2.50
 基準表項目ID：shulin.regional.funeral_facility</t>
       </text>
     </comment>
@@ -9431,7 +9431,7 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±25.0%、級距6.25%；(3−4)×6.25 = +6.25</t>
+          <t>查表：共5級、最大±25.0%、級距6.25%；(4−3)×6.25 = +6.25</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="F95" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±15.0%、級距3.75%；(1−5)×3.75 = +15.00</t>
+          <t>查表：共5級、最大±15.0%、級距3.75%；(5−1)×3.75 = +15.00</t>
         </is>
       </c>
       <c r="G95" s="0" t="inlineStr">
@@ -10897,7 +10897,7 @@
       </c>
       <c r="F98" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±15.0%、級距3.75%；(1−4)×3.75 = +11.25</t>
+          <t>查表：共5級、最大±15.0%、級距3.75%；(4−1)×3.75 = +11.25</t>
         </is>
       </c>
       <c r="G98" s="0" t="inlineStr">
@@ -11019,7 +11019,7 @@
       </c>
       <c r="F101" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±15.0%、級距3.75%；(1−4)×3.75 = +11.25</t>
+          <t>查表：共5級、最大±15.0%、級距3.75%；(4−1)×3.75 = +11.25</t>
         </is>
       </c>
       <c r="G101" s="0" t="inlineStr">
@@ -11223,7 +11223,7 @@
       </c>
       <c r="F106" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±12.0%、級距3.0%；(3−5)×3.0 = +6.00</t>
+          <t>查表：共5級、最大±12.0%、級距3.0%；(5−3)×3.0 = +6.00</t>
         </is>
       </c>
       <c r="G106" s="0" t="inlineStr">
@@ -11345,7 +11345,7 @@
       </c>
       <c r="F109" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±12.0%、級距3.0%；(3−5)×3.0 = +6.00</t>
+          <t>查表：共5級、最大±12.0%、級距3.0%；(5−3)×3.0 = +6.00</t>
         </is>
       </c>
       <c r="G109" s="0" t="inlineStr">
@@ -11467,7 +11467,7 @@
       </c>
       <c r="F112" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±12.0%、級距3.0%；(3−5)×3.0 = +6.00</t>
+          <t>查表：共5級、最大±12.0%、級距3.0%；(5−3)×3.0 = +6.00</t>
         </is>
       </c>
       <c r="G112" s="0" t="inlineStr">
@@ -11671,7 +11671,7 @@
       </c>
       <c r="F117" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±10.0%、級距2.5%；(2−1)×2.5 = -2.50</t>
+          <t>查表：共5級、最大±10.0%、級距2.5%；(1−2)×2.5 = -2.50</t>
         </is>
       </c>
       <c r="G117" s="0" t="inlineStr">
@@ -12363,7 +12363,7 @@
       </c>
       <c r="F134" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±4.0%、級距1.0%；(1−2)×1.0 = +1.00</t>
+          <t>查表：共5級、最大±4.0%、級距1.0%；(2−1)×1.0 = +1.00</t>
         </is>
       </c>
       <c r="G134" s="0" t="inlineStr">
@@ -12811,7 +12811,7 @@
       </c>
       <c r="F145" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±4.0%、級距1.0%；(4−5)×1.0 = +1.00</t>
+          <t>查表：共5級、最大±4.0%、級距1.0%；(5−4)×1.0 = +1.00</t>
         </is>
       </c>
       <c r="G145" s="0" t="inlineStr">
@@ -13015,7 +13015,7 @@
       </c>
       <c r="F150" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±10.0%、級距2.5%；(2−3)×2.5 = +2.50</t>
+          <t>查表：共5級、最大±10.0%、級距2.5%；(3−2)×2.5 = +2.50</t>
         </is>
       </c>
       <c r="G150" s="0" t="inlineStr">
@@ -13137,7 +13137,7 @@
       </c>
       <c r="F153" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±10.0%、級距2.5%；(2−1)×2.5 = -2.50</t>
+          <t>查表：共5級、最大±10.0%、級距2.5%；(1−2)×2.5 = -2.50</t>
         </is>
       </c>
       <c r="G153" s="0" t="inlineStr">
@@ -13259,7 +13259,7 @@
       </c>
       <c r="F156" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±10.0%、級距2.5%；(2−1)×2.5 = -2.50</t>
+          <t>查表：共5級、最大±10.0%、級距2.5%；(1−2)×2.5 = -2.50</t>
         </is>
       </c>
       <c r="G156" s="0" t="inlineStr">
@@ -16599,7 +16599,7 @@
       </c>
       <c r="F238" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±8.0%、級距2.0%；(3−1)×2.0 = -4.00</t>
+          <t>查表：共5級、最大±8.0%、級距2.0%；(1−3)×2.0 = -4.00</t>
         </is>
       </c>
       <c r="G238" s="0" t="inlineStr">
@@ -16721,7 +16721,7 @@
       </c>
       <c r="F241" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±8.0%、級距2.0%；(3−1)×2.0 = -4.00</t>
+          <t>查表：共5級、最大±8.0%、級距2.0%；(1−3)×2.0 = -4.00</t>
         </is>
       </c>
       <c r="G241" s="0" t="inlineStr">
@@ -16843,7 +16843,7 @@
       </c>
       <c r="F244" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±8.0%、級距2.0%；(3−2)×2.0 = -2.00</t>
+          <t>查表：共5級、最大±8.0%、級距2.0%；(2−3)×2.0 = -2.00</t>
         </is>
       </c>
       <c r="G244" s="0" t="inlineStr">
@@ -17291,7 +17291,7 @@
       </c>
       <c r="F255" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±8.0%、級距2.0%；(1−3)×2.0 = +4.00</t>
+          <t>查表：共5級、最大±8.0%、級距2.0%；(3−1)×2.0 = +4.00</t>
         </is>
       </c>
       <c r="G255" s="0" t="inlineStr">
@@ -17495,7 +17495,7 @@
       </c>
       <c r="F260" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50</t>
+          <t>查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50</t>
         </is>
       </c>
       <c r="G260" s="0" t="inlineStr">
@@ -17617,7 +17617,7 @@
       </c>
       <c r="F263" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50</t>
+          <t>查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50</t>
         </is>
       </c>
       <c r="G263" s="0" t="inlineStr">
@@ -17739,7 +17739,7 @@
       </c>
       <c r="F266" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50</t>
+          <t>查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50</t>
         </is>
       </c>
       <c r="G266" s="0" t="inlineStr">
@@ -17943,7 +17943,7 @@
       </c>
       <c r="F271" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50</t>
+          <t>查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50</t>
         </is>
       </c>
       <c r="G271" s="0" t="inlineStr">
@@ -18065,7 +18065,7 @@
       </c>
       <c r="F274" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±6.0%、級距1.5%；(1−2)×1.5 = +1.50</t>
+          <t>查表：共5級、最大±6.0%、級距1.5%；(2−1)×1.5 = +1.50</t>
         </is>
       </c>
       <c r="G274" s="0" t="inlineStr">
@@ -19287,7 +19287,7 @@
       </c>
       <c r="F304" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±10.0%、級距2.5%；(5−4)×2.5 = -2.50</t>
+          <t>查表：共5級、最大±10.0%、級距2.5%；(4−5)×2.5 = -2.50</t>
         </is>
       </c>
       <c r="G304" s="0" t="inlineStr">
@@ -19531,7 +19531,7 @@
       </c>
       <c r="F310" s="0" t="inlineStr">
         <is>
-          <t>查表：共5級、最大±10.0%、級距2.5%；(5−4)×2.5 = -2.50</t>
+          <t>查表：共5級、最大±10.0%、級距2.5%；(4−5)×2.5 = -2.50</t>
         </is>
       </c>
       <c r="G310" s="0" t="inlineStr">

</xml_diff>